<commit_message>
Update time/materials, place onshape link
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_AspenBoler.xlsx
+++ b/Documentation/Contributions/TimeReport_AspenBoler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19042\Downloads\HW\CEN4908\plant-partner\Documentation\Contributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{571C2E69-5314-41D6-9E56-2CBB4E5F5FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDDF59EA-DDD8-46AA-9D5F-38D6F1E9D774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{605B5A91-C2DF-4ED5-9E2C-366EB894E8F1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="91">
   <si>
     <t>Name:</t>
   </si>
@@ -302,10 +302,13 @@
     <t>Discussed what needed to be done and assigned tasks regarding NPK and PCB; Talked through 3D and decided on what structures to go through with; set up documentation and delegated when and who needed to complete what</t>
   </si>
   <si>
-    <t>Check-in 9: Met with tyler to show integration of current databse changes into main, communication error handling, NPK integration, the current arrival and soldering of the new PCB, and the plans for the 3D printed housing.</t>
-  </si>
-  <si>
     <t>Tested NPK sensor and confirmed it worked with integrated main code. Then proceeded to complete Beta Tests notes.</t>
+  </si>
+  <si>
+    <t>Worked on onshape design</t>
+  </si>
+  <si>
+    <t>Check-in 9: Met with tyler to show integration of current database changes into main, communication error handling, NPK integration, the current arrival and soldering of the new PCB, and the plans for the 3D printed housing.</t>
   </si>
 </sst>
 </file>
@@ -900,7 +903,7 @@
       </c>
       <c r="E1" s="6">
         <f>SUM(E4:E199)</f>
-        <v>5.9493055555555552</v>
+        <v>6.2270833333333329</v>
       </c>
       <c r="F1" s="15"/>
     </row>
@@ -2329,7 +2332,7 @@
         <v>1.388888888888884E-2</v>
       </c>
       <c r="F70" s="13" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
@@ -2350,30 +2353,50 @@
         <v>5.4861111111111138E-2</v>
       </c>
       <c r="F71" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="7">
+        <v>46094</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C72" s="17">
+        <v>0.78472222222222221</v>
+      </c>
+      <c r="D72" s="17">
+        <v>0.90625</v>
+      </c>
+      <c r="E72" s="10">
+        <f t="shared" si="1"/>
+        <v>0.12152777777777779</v>
+      </c>
+      <c r="F72" s="13" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="7"/>
-      <c r="B72" s="8"/>
-      <c r="C72" s="17"/>
-      <c r="D72" s="17"/>
-      <c r="E72" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F72" s="13"/>
-    </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="7"/>
-      <c r="B73" s="8"/>
-      <c r="C73" s="17"/>
-      <c r="D73" s="17"/>
+      <c r="A73" s="7">
+        <v>46095</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C73" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="D73" s="17">
+        <v>0.65625</v>
+      </c>
       <c r="E73" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="F73" s="13"/>
+        <v>0.15625</v>
+      </c>
+      <c r="F73" s="13" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="7"/>

</xml_diff>

<commit_message>
Update end time and pinouts
</commit_message>
<xml_diff>
--- a/Documentation/Contributions/TimeReport_AspenBoler.xlsx
+++ b/Documentation/Contributions/TimeReport_AspenBoler.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\19042\Downloads\HW\CEN4908\plant-partner\Documentation\Contributions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F124C94-9E74-4943-8A54-B7236E18E6A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834B134F-6F73-4E80-9B1E-AD4DD8898AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{605B5A91-C2DF-4ED5-9E2C-366EB894E8F1}"/>
   </bookViews>
@@ -320,7 +320,7 @@
     <t>Fixing onshape design</t>
   </si>
   <si>
-    <t>Helped merge and fix inconsistied encountered with new handshake protocols and app.</t>
+    <t>Helped merge and fix inconsistied encountered with new handshake protocols and app., test PCB, adjusted 3D model to fit printer</t>
   </si>
 </sst>
 </file>
@@ -915,7 +915,7 @@
       </c>
       <c r="E1" s="6">
         <f>SUM(E4:E199)</f>
-        <v>6.2361111111111089</v>
+        <v>6.8979166666666645</v>
       </c>
       <c r="F1" s="15"/>
     </row>
@@ -2525,10 +2525,12 @@
       <c r="C79" s="17">
         <v>0.44444444444444442</v>
       </c>
-      <c r="D79" s="17"/>
+      <c r="D79" s="17">
+        <v>0.66180555555555554</v>
+      </c>
       <c r="E79" s="10">
         <f t="shared" si="1"/>
-        <v>-0.44444444444444442</v>
+        <v>0.21736111111111112</v>
       </c>
       <c r="F79" s="13" t="s">
         <v>94</v>

</xml_diff>